<commit_message>
feat: :sparkles: Added the chromedriver.exe, so it can be used in a .exe
</commit_message>
<xml_diff>
--- a/datos_cuentas.xlsx
+++ b/datos_cuentas.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Cuenta creada y unida a la sección correctamente.</t>
+          <t>Cuenta creada y unida a la sección.</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Cuenta creada y unida a la sección correctamente.</t>
+          <t>Cuenta creada y unida a la sección.</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Cuenta creada y unida a la sección correctamente.</t>
+          <t>Cuenta creada y unida a la sección.</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Cuenta creada y unida a la sección correctamente.</t>
+          <t>Cuenta creada y unida a la sección.</t>
         </is>
       </c>
     </row>

</xml_diff>